<commit_message>
Retire FRCoreInterpretationExtension de ServiceRequest
Une demande d'acte/d'examen n'a pas de notion d'interprétation
(celle-ci s'applique au résultat, pas à la demande). 2d1361864f5c5fc8e68bf318cac1f9036ff86306
</commit_message>
<xml_diff>
--- a/nr-doc-core-service-request/ig/StructureDefinition-fr-core-method-extension.xlsx
+++ b/nr-doc-core-service-request/ig/StructureDefinition-fr-core-method-extension.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-22T07:18:24+00:00</t>
+    <t>2026-07-23T09:21:02+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -350,7 +350,7 @@
     <t>required</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-hl7-v3-ObservationMethod-cisis|20260420150249</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-hl7-v3-ObservationMethod-cisis|20260619134042</t>
   </si>
   <si>
     <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}

</xml_diff>